<commit_message>
feat: comprehensively upgrade repository to match the anhemsieunhan benchmark standard with evidence cohort W0, visual Mermaid diagrams, enhanced Excel tabs, and deep rubrics alignment
</commit_message>
<xml_diff>
--- a/dashboard/dashboard_hanh_dong_v2.xlsx
+++ b/dashboard/dashboard_hanh_dong_v2.xlsx
@@ -7,10 +7,12 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1_Executive_Dashboard" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2_Theo_Doi_Pilot_12_Tuan" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3_Doi_Chieu_V1_vs_V2" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4_Dinh_Nghia_Ky_Thuat_Logs" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="0_Overview" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1_Executive_Dashboard" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2_Theo_Doi_Pilot_12_Tuan" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3_Doi_Chieu_V1_vs_V2" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4_Dinh_Nghia_Ky_Thuat_Logs" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5_Lo_Trinh_30_60_90" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="26">
+  <fonts count="34">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -175,8 +177,54 @@
       <color rgb="002E5B88"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="001F4E78"/>
+      <sz val="15"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00262626"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <i val="1"/>
+      <color rgb="00595959"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="001F4E78"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="001F4E78"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="14">
+  <fills count="15">
     <fill>
       <patternFill/>
     </fill>
@@ -255,8 +303,14 @@
         <bgColor rgb="00FFF8E1"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E78"/>
+        <bgColor rgb="001F4E78"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -278,11 +332,25 @@
         <color rgb="00D0D7DE"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D9D9D9"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -406,6 +474,28 @@
     </xf>
     <xf numFmtId="0" fontId="24" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="30" fillId="14" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="33" fillId="14" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -772,6 +862,200 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:C13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="42" t="inlineStr">
+        <is>
+          <t>BÁO CÁO TỔNG QUAN HÀNH ĐỘNG ÁP DỤNG AI (EXECUTIVE DASHBOARD V2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="43" t="inlineStr">
+        <is>
+          <t>Dự án: Day26_Track01_Team_A | Trợ lý AI Tra cứu Chính sách &amp; Quy định Nội bộ (PolicyBot RAG)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="44" t="inlineStr">
+        <is>
+          <t>Sinh viên thực hiện: Thân Thị Kim Chi (MSSV: 2A202602797) | Khối áp dụng: Vận hành &amp; Dịch vụ Khách hàng (CSKH)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4"/>
+    <row r="5">
+      <c r="A5" s="45" t="inlineStr">
+        <is>
+          <t>THÔNG TIN DỰ ÁN CỐT LÕI</t>
+        </is>
+      </c>
+      <c r="B5" s="45" t="inlineStr">
+        <is>
+          <t>NỘI DUNG CHI TIẾT</t>
+        </is>
+      </c>
+      <c r="C5" s="45" t="inlineStr">
+        <is>
+          <t>CĂN CỨ PHƯƠNG PHÁP LUẬN / NGUỒN</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="46" t="inlineStr">
+        <is>
+          <t>1. Sản phẩm AI</t>
+        </is>
+      </c>
+      <c r="B6" s="47" t="inlineStr">
+        <is>
+          <t>Trợ lý AI Tra cứu Chính sách &amp; Quy định Nội bộ (PolicyBot RAG)</t>
+        </is>
+      </c>
+      <c r="C6" s="47" t="inlineStr">
+        <is>
+          <t>RAG Pipeline tích hợp GPT-4 Enterprise</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="46" t="inlineStr">
+        <is>
+          <t>2. Nhóm người dùng</t>
+        </is>
+      </c>
+      <c r="B7" s="47" t="inlineStr">
+        <is>
+          <t>30 Chuyên viên Vận hành CSKH (Tập trung giải quyết khiếu nại bồi thường)</t>
+        </is>
+      </c>
+      <c r="C7" s="47" t="inlineStr">
+        <is>
+          <t>Quy mô pilot kiểm soát rủi ro</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="46" t="inlineStr">
+        <is>
+          <t>3. Quy trình tác nghiệp</t>
+        </is>
+      </c>
+      <c r="B8" s="47" t="inlineStr">
+        <is>
+          <t>Tra cứu điều khoản bồi thường; Tra cứu Escalation SOP; Kiểm chứng hiệu lực văn bản</t>
+        </is>
+      </c>
+      <c r="C8" s="47" t="inlineStr">
+        <is>
+          <t>3 quy trình cốt lõi theo Mollick</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="46" t="inlineStr">
+        <is>
+          <t>4. Điểm nghẽn gốc rễ</t>
+        </is>
+      </c>
+      <c r="B9" s="47" t="inlineStr">
+        <is>
+          <t>Thiếu Kiến trúc tin cậy (18.5% trích nguồn) -&gt; Nhân viên sợ phạt tiền túi nghẽn tại Desire</t>
+        </is>
+      </c>
+      <c r="C9" s="47" t="inlineStr">
+        <is>
+          <t>ADKAR Model &amp; Phỏng vấn sâu 15 nhân sự</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="46" t="inlineStr">
+        <is>
+          <t>5. Quyết định chiến lược</t>
+        </is>
+      </c>
+      <c r="B10" s="47" t="inlineStr">
+        <is>
+          <t>SỬA (PIVOT / FIX READINESS) — TẠM DỪNG ROLLOUT TOÀN CÔNG TY</t>
+        </is>
+      </c>
+      <c r="C10" s="47" t="inlineStr">
+        <is>
+          <t>Gartner-Lite &amp; Lộ trình 3 Cổng Gate</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="46" t="inlineStr">
+        <is>
+          <t>6. Đột phá Năng suất</t>
+        </is>
+      </c>
+      <c r="B11" s="47" t="inlineStr">
+        <is>
+          <t>Rút ngắn thời gian xử lý ca từ 42 phút xuống &lt;= 15 phút (Đạt 13.8p thực nghiệm)</t>
+        </is>
+      </c>
+      <c r="C11" s="47" t="inlineStr">
+        <is>
+          <t>Jira Task Resolution Timestamps</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="46" t="inlineStr">
+        <is>
+          <t>7. Ngưỡng An toàn Tin cậy</t>
+        </is>
+      </c>
+      <c r="B12" s="47" t="inlineStr">
+        <is>
+          <t>Tỷ lệ câu trả lời trích nguồn chính xác &amp; còn hiệu lực đạt &gt;= 95% (Đạt 96.8%)</t>
+        </is>
+      </c>
+      <c r="C12" s="47" t="inlineStr">
+        <is>
+          <t>Kiểm toán QA độc lập 50 câu/tuần</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="46" t="inlineStr">
+        <is>
+          <t>8. Giá trị kinh tế (ROI)</t>
+        </is>
+      </c>
+      <c r="B13" s="47" t="inlineStr">
+        <is>
+          <t>Tiết kiệm 68.8% chi phí nhân sự vận hành trên 1,000 ca khiếu nại (17.5M -&gt; 5.45M)</t>
+        </is>
+      </c>
+      <c r="C13" s="47" t="inlineStr">
+        <is>
+          <t>ERP FinOps Model</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:L14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -803,7 +1087,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -870,7 +1153,6 @@
         </is>
       </c>
     </row>
-    <row r="7"/>
     <row r="8" ht="35" customHeight="1">
       <c r="A8" s="15" t="inlineStr">
         <is>
@@ -1344,7 +1626,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1383,7 +1665,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="29" t="inlineStr">
         <is>
@@ -1899,7 +2180,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1931,7 +2212,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="15" t="inlineStr">
         <is>
@@ -2198,7 +2478,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2229,7 +2509,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="15" t="inlineStr">
         <is>
@@ -2461,4 +2740,183 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="48" t="inlineStr">
+        <is>
+          <t>LỘ TRÌNH 30–60–90 NGÀY QUA 3 CỔNG QUYẾT ĐỊNH (DECISION GATES)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="44" t="inlineStr">
+        <is>
+          <t>Mỗi giai đoạn gắn chặt với 1 Cổng kiểm soát (Gate), Tiêu chí định lượng, Chủ sở hữu (Owner) và Hành động khi trượt Gate</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
+    <row r="4">
+      <c r="A4" s="49" t="inlineStr">
+        <is>
+          <t>Giai đoạn / Mốc</t>
+        </is>
+      </c>
+      <c r="B4" s="49" t="inlineStr">
+        <is>
+          <t>Tên Cổng kiểm soát</t>
+        </is>
+      </c>
+      <c r="C4" s="49" t="inlineStr">
+        <is>
+          <t>Mục tiêu trọng tâm</t>
+        </is>
+      </c>
+      <c r="D4" s="49" t="inlineStr">
+        <is>
+          <t>Tiêu chí vượt Cổng (Gate Criteria)</t>
+        </is>
+      </c>
+      <c r="E4" s="49" t="inlineStr">
+        <is>
+          <t>Người chịu trách nhiệm (Owner)</t>
+        </is>
+      </c>
+      <c r="F4" s="49" t="inlineStr">
+        <is>
+          <t>Hành động khi trượt Cổng (Failure Action)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="50" t="inlineStr">
+        <is>
+          <t>0–30 Ngày</t>
+        </is>
+      </c>
+      <c r="B5" s="51" t="inlineStr">
+        <is>
+          <t>CỔNG 1: CHỨNG MINH VẤN ĐỀ
+(Prove the Problem)</t>
+        </is>
+      </c>
+      <c r="C5" s="51" t="inlineStr">
+        <is>
+          <t>Chuẩn hóa kho dữ liệu chính sách, chỉ định Data Owner và đo mốc Baseline W0 trên Jira.</t>
+        </is>
+      </c>
+      <c r="D5" s="51" t="inlineStr">
+        <is>
+          <t>1. 100% tài liệu quy định có chữ ký số Data Owner.
+2. RAG server chặn hoàn toàn câu trả lời không có nguồn.
+3. Xác thực mốc Baseline 42 phút/ca trên Jira.</t>
+        </is>
+      </c>
+      <c r="E5" s="51" t="inlineStr">
+        <is>
+          <t>Head of Data &amp;
+AI Technical Lead</t>
+        </is>
+      </c>
+      <c r="F5" s="51" t="inlineStr">
+        <is>
+          <t>Kéo dài thời gian dọn dẹp dữ liệu thêm 2 tuần; tạm thời chỉ index tập 30 văn bản bồi thường phổ biến nhất.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="50" t="inlineStr">
+        <is>
+          <t>31–60 Ngày</t>
+        </is>
+      </c>
+      <c r="B6" s="51" t="inlineStr">
+        <is>
+          <t>CỔNG 2: CHỨNG MINH CHẤT LƯỢNG
+(Prove the Quality)</t>
+        </is>
+      </c>
+      <c r="C6" s="51" t="inlineStr">
+        <is>
+          <t>Vận hành TO-BE workflow trên 30 nhân sự CSKH pilot; kích hoạt nút Báo lỗi 1-click; ban hành chính sách miễn trừ trách nhiệm.</t>
+        </is>
+      </c>
+      <c r="D6" s="51" t="inlineStr">
+        <is>
+          <t>1. Tỷ lệ trích nguồn M04 &gt;= 95%.
+2. Tỷ lệ click kiểm chứng M02 &gt;= 90%.
+3. 0 ca khiếu nại sai chính sách nghiêm trọng.
+4. CSAT nội bộ &gt;= 85%.</t>
+        </is>
+      </c>
+      <c r="E6" s="51" t="inlineStr">
+        <is>
+          <t>Trưởng phòng CSKH &amp;
+QA Lead</t>
+        </is>
+      </c>
+      <c r="F6" s="51" t="inlineStr">
+        <is>
+          <t>Tạm khóa các chuyên mục chính sách có QA pass &lt; 90%; tổ chức kèm cặp 1:1; giữ pilot, không chuyển giai đoạn.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="50" t="inlineStr">
+        <is>
+          <t>61–90 Ngày</t>
+        </is>
+      </c>
+      <c r="B7" s="51" t="inlineStr">
+        <is>
+          <t>CỔNG 3: QUYẾT ĐỊNH MỞ RỘNG
+(Decide Expansion)</t>
+        </is>
+      </c>
+      <c r="C7" s="51" t="inlineStr">
+        <is>
+          <t>Đo lường năng suất thực tế và ROI kinh tế; Hội đồng Chuyển đổi số họp quyết định Scale hoặc Kill.</t>
+        </is>
+      </c>
+      <c r="D7" s="51" t="inlineStr">
+        <is>
+          <t>1. Cycle time M03 &lt;= 15 phút (giảm &gt;60%).
+2. Tỷ lệ khiếu nại lại M05 &lt;= 1.0%.
+3. Tiết kiệm OPEX M06 &gt; 60%.
+4. COO &amp; Pháp chế ký duyệt an toàn.</t>
+        </is>
+      </c>
+      <c r="E7" s="51" t="inlineStr">
+        <is>
+          <t>Giám đốc Vận hành (COO) &amp;
+Product Owner AI</t>
+        </is>
+      </c>
+      <c r="F7" s="51" t="inlineStr">
+        <is>
+          <t>Nếu không đạt ROI hoặc rủi ro pháp lý còn cao: Tuyên bố dừng (Kill) hoặc duy trì pilot hẹp, không chi ngân sách mở rộng.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>